<commit_message>
verify is username or user email is already used
</commit_message>
<xml_diff>
--- a/App/CLI-backend/databases/UserDatabase.xlsx
+++ b/App/CLI-backend/databases/UserDatabase.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent>
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DELL\Downloads\ZTH-Team-Deltaspace\App\CLI-backend\databases\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\serba\AppData\Roaming\SPB_Data\ZTH-Team-Deltaspace\App\CLI-backend\databases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A1F3EA5-F442-48DD-B2EE-08EDFCB886DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADF3B014-C8E1-4E5F-83CB-3E4AECC90F02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2988" yWindow="2100" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet0" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="33">
   <si>
     <t>ID</t>
   </si>
@@ -80,6 +80,45 @@
   </si>
   <si>
     <t>15-02-2000</t>
+  </si>
+  <si>
+    <t>$2a$12$kwjwLDgW5.yyK5l0bDbO3uUawRc.77RQZ1eZ32bmC1jIV1EIOhV9a</t>
+  </si>
+  <si>
+    <t>$2a$12$9YTuoKj6bZmyR7pHTZbAL.FZC7D/7xpxliPps4loZAAXLgUk5Q576</t>
+  </si>
+  <si>
+    <t>$2a$12$d4LQ0bY8aipPIDXmS0qnLOZuPWaLXLHnRdUhnu/N5pHnMzYoR3rwW</t>
+  </si>
+  <si>
+    <t>Serban123</t>
+  </si>
+  <si>
+    <t>s@y.com</t>
+  </si>
+  <si>
+    <t>$2a$12$WBL81iGG3XPCx9gH7hPJRe7edY2DPDJnBAviD6/n/IFPJ02UGgU3a</t>
+  </si>
+  <si>
+    <t>30-08-2000</t>
+  </si>
+  <si>
+    <t>$2a$12$mQxp63of/TPVUOx.IVzlWOhGBwl5ZcfpjEoLkzYS4CDebjHGHoP42</t>
+  </si>
+  <si>
+    <t>$2a$12$4Bw4NdHXJ.1ed2X/Jnz3X.n3CobsQt35EA6Mu0qVSNoWbD7sCRbeq</t>
+  </si>
+  <si>
+    <t>$2a$12$pcwaVErtO8XzrBU8aktfL.hA.xRE/Z9vVkoDAZf1l11R8rsCsiFny</t>
+  </si>
+  <si>
+    <t>$2a$12$FwGNUQoxjSsE9o9N0xxTOuChOhjb8GVkhFz7rqX3TgWqwU1rDVFtq</t>
+  </si>
+  <si>
+    <t>$2a$12$vgVwZl.BhCbITo8JEFu4zOuIgzO/XIcyglbh9QRjxomiTn8m0EX6e</t>
+  </si>
+  <si>
+    <t>$2a$12$0CdrxqVbob0qzfT3peq7buGqy4bU7o0.J4b3UHDHN.fc4Oou2hUle</t>
   </si>
 </sst>
 </file>
@@ -452,17 +491,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:E14"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" bestFit="true" customWidth="true" width="2.7109375"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="9.20703125"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="9.7109375"/>
     <col min="3" max="3" bestFit="true" customWidth="true" width="22.92578125"/>
     <col min="4" max="4" bestFit="true" customWidth="true" width="66.76171875"/>
     <col min="5" max="5" bestFit="true" customWidth="true" width="10.91015625"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s" s="0">
         <v>0</v>
       </c>
@@ -479,7 +518,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" t="s" s="0">
         <v>5</v>
       </c>
@@ -496,7 +535,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" t="s" s="0">
         <v>10</v>
       </c>
@@ -513,7 +552,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" t="s" s="0">
         <v>15</v>
       </c>
@@ -528,6 +567,176 @@
       </c>
       <c r="E4" t="s" s="0">
         <v>19</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A5" t="s" s="0">
+        <v>5</v>
+      </c>
+      <c r="B5" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="C5" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="D5" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="E5" t="s" s="0">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A6" t="s" s="0">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="C6" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="D6" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="E6" t="s" s="0">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A7" t="s" s="0">
+        <v>5</v>
+      </c>
+      <c r="B7" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="C7" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="D7" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="E7" t="s" s="0">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A8" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="B8" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="C8" t="s" s="0">
+        <v>24</v>
+      </c>
+      <c r="D8" t="s" s="0">
+        <v>25</v>
+      </c>
+      <c r="E8" t="s" s="0">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A9" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="B9" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="C9" t="s" s="0">
+        <v>24</v>
+      </c>
+      <c r="D9" t="s" s="0">
+        <v>27</v>
+      </c>
+      <c r="E9" t="s" s="0">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A10" t="s" s="0">
+        <v>5</v>
+      </c>
+      <c r="B10" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="C10" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="D10" t="s" s="0">
+        <v>28</v>
+      </c>
+      <c r="E10" t="s" s="0">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s" s="0">
+        <v>5</v>
+      </c>
+      <c r="B11" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="C11" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="D11" t="s" s="0">
+        <v>29</v>
+      </c>
+      <c r="E11" t="s" s="0">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s" s="0">
+        <v>5</v>
+      </c>
+      <c r="B12" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="C12" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="D12" t="s" s="0">
+        <v>30</v>
+      </c>
+      <c r="E12" t="s" s="0">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s" s="0">
+        <v>5</v>
+      </c>
+      <c r="B13" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="C13" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="D13" t="s" s="0">
+        <v>31</v>
+      </c>
+      <c r="E13" t="s" s="0">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s" s="0">
+        <v>5</v>
+      </c>
+      <c r="B14" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="C14" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="D14" t="s" s="0">
+        <v>32</v>
+      </c>
+      <c r="E14" t="s" s="0">
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
check email and user duplicates v2
</commit_message>
<xml_diff>
--- a/App/CLI-backend/databases/UserDatabase.xlsx
+++ b/App/CLI-backend/databases/UserDatabase.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="43">
   <si>
     <t>ID</t>
   </si>
@@ -119,6 +119,36 @@
   </si>
   <si>
     <t>$2a$12$0CdrxqVbob0qzfT3peq7buGqy4bU7o0.J4b3UHDHN.fc4Oou2hUle</t>
+  </si>
+  <si>
+    <t>$2a$12$DKf0QJLMBsE1Hdsq7sTlWuqlqebw247P7lH9t1u.HaZZ6hv7uAHLq</t>
+  </si>
+  <si>
+    <t>$2a$12$iWKkKScGPqA8Ln6o4sezpOjUMhK47jflt66brWmljrkA.zogYfjCa</t>
+  </si>
+  <si>
+    <t>$2a$12$eXiy.07Cy.vq/f7xSvMvEupq99A7KNl3UxFt8tIyp5UdmWgiY2/KW</t>
+  </si>
+  <si>
+    <t>$2a$12$mEoXZJq.yRsJjs2XwuABleUVs8sF/ye6I6WLeh06PcqhZvUQLplL6</t>
+  </si>
+  <si>
+    <t>$2a$12$dTuY0JowgNNg6oFHk2xxH.ZJKBEsyVD/XTrUUH88drkYPussFgzeC</t>
+  </si>
+  <si>
+    <t>$2a$12$7crWFGlGwUf2qLXNVOLKBemQ0VWDnTi06MnXdXQrEyMkrVuPTPwCS</t>
+  </si>
+  <si>
+    <t>Serban12</t>
+  </si>
+  <si>
+    <t>s@y1.com</t>
+  </si>
+  <si>
+    <t>$2a$12$lL2Vd/OdYOnVOgcDtcy1Be.m5sHYA9jC.BAvwrQy9G.L0VuphvOJ6</t>
+  </si>
+  <si>
+    <t>30-07-2004</t>
   </si>
 </sst>
 </file>
@@ -491,13 +521,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" bestFit="true" customWidth="true" width="2.7109375"/>
     <col min="2" max="2" bestFit="true" customWidth="true" width="9.7109375"/>
     <col min="3" max="3" bestFit="true" customWidth="true" width="22.92578125"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="66.76171875"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="67.06640625"/>
     <col min="5" max="5" bestFit="true" customWidth="true" width="10.91015625"/>
   </cols>
   <sheetData>
@@ -739,6 +769,125 @@
         <v>9</v>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="s" s="0">
+        <v>5</v>
+      </c>
+      <c r="B15" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="C15" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="D15" t="s" s="0">
+        <v>33</v>
+      </c>
+      <c r="E15" t="s" s="0">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s" s="0">
+        <v>5</v>
+      </c>
+      <c r="B16" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="C16" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="D16" t="s" s="0">
+        <v>34</v>
+      </c>
+      <c r="E16" t="s" s="0">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s" s="0">
+        <v>5</v>
+      </c>
+      <c r="B17" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="C17" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="D17" t="s" s="0">
+        <v>35</v>
+      </c>
+      <c r="E17" t="s" s="0">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="s" s="0">
+        <v>5</v>
+      </c>
+      <c r="B18" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="C18" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="D18" t="s" s="0">
+        <v>36</v>
+      </c>
+      <c r="E18" t="s" s="0">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="s" s="0">
+        <v>5</v>
+      </c>
+      <c r="B19" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="C19" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="D19" t="s" s="0">
+        <v>37</v>
+      </c>
+      <c r="E19" t="s" s="0">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="s" s="0">
+        <v>5</v>
+      </c>
+      <c r="B20" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="C20" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="D20" t="s" s="0">
+        <v>38</v>
+      </c>
+      <c r="E20" t="s" s="0">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="B21" t="s" s="0">
+        <v>39</v>
+      </c>
+      <c r="C21" t="s" s="0">
+        <v>40</v>
+      </c>
+      <c r="D21" t="s" s="0">
+        <v>41</v>
+      </c>
+      <c r="E21" t="s" s="0">
+        <v>42</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
UserId increments correctly now.
</commit_message>
<xml_diff>
--- a/App/CLI-backend/databases/UserDatabase.xlsx
+++ b/App/CLI-backend/databases/UserDatabase.xlsx
@@ -3,12 +3,12 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <mc:AlternateContent>
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DELL\Downloads\ZTH-Team-Deltaspace\App\CLI-backend\databases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80DA16A1-D919-4849-A6DB-CC71D870E10E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{798B4254-7D9D-4FBA-9192-C9BA1ECBDA82}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
   <si>
     <t>ID</t>
   </si>
@@ -35,12 +35,43 @@
   </si>
   <si>
     <t>Date of Birth</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>admin</t>
+  </si>
+  <si>
+    <t>test@admin</t>
+  </si>
+  <si>
+    <t>$2a$12$DDjfx2JAW.3U4n4HNJe/SO5WQTfFlLsmoN0bfb5I9aNKRDXBVVfzS</t>
+  </si>
+  <si>
+    <t>01-01-2000</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>Mihai14</t>
+  </si>
+  <si>
+    <t>mihai@gmail.com</t>
+  </si>
+  <si>
+    <t>$2a$12$AomzYMZwq2MjzsPAN9kK3OM6OheRkKWP/FSsBfbCDMiWqxvixmn1.</t>
+  </si>
+  <si>
+    <t>11-09-1100</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="0"/>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -406,31 +437,65 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="2.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="64.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="2.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="9.20703125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="15.23046875"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="65.36328125"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="10.91015625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+      <c r="A1" t="s" s="0">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" t="s" s="0">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" t="s" s="0">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" t="s" s="0">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" t="s" s="0">
         <v>4</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="0">
+        <v>5</v>
+      </c>
+      <c r="B2" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="C2" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="D2" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="E2" t="s" s="0">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="B3" t="s" s="0">
+        <v>11</v>
+      </c>
+      <c r="C3" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="D3" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="E3" t="s" s="0">
+        <v>14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Finished UserDatabse writing proccess
</commit_message>
<xml_diff>
--- a/App/CLI-backend/databases/UserDatabase.xlsx
+++ b/App/CLI-backend/databases/UserDatabase.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DELL\Downloads\ZTH-Team-Deltaspace\App\CLI-backend\databases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{798B4254-7D9D-4FBA-9192-C9BA1ECBDA82}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD3AA2ED-248E-4D19-BB1F-F5DC9E904FFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="19">
   <si>
     <t>ID</t>
   </si>
@@ -46,7 +46,7 @@
     <t>test@admin</t>
   </si>
   <si>
-    <t>$2a$12$DDjfx2JAW.3U4n4HNJe/SO5WQTfFlLsmoN0bfb5I9aNKRDXBVVfzS</t>
+    <t>$2a$12$.8f5of5jHYP0IkiHyRvaB.fNCEVGKTM2ZgjeuF/Jd1IVfwFDft0pS</t>
   </si>
   <si>
     <t>01-01-2000</t>
@@ -58,13 +58,25 @@
     <t>Mihai14</t>
   </si>
   <si>
-    <t>mihai@gmail.com</t>
-  </si>
-  <si>
-    <t>$2a$12$AomzYMZwq2MjzsPAN9kK3OM6OheRkKWP/FSsBfbCDMiWqxvixmn1.</t>
-  </si>
-  <si>
-    <t>11-09-1100</t>
+    <t>mihaiviorelstan@gmail.com</t>
+  </si>
+  <si>
+    <t>$2a$12$dFXj26exmWO1qy1T8a2BJO1WUG5Bx808hZ.bWQBValcptUoiJYIYu</t>
+  </si>
+  <si>
+    <t>15-05-2004</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>Mihai12</t>
+  </si>
+  <si>
+    <t>mihaiviis@gmail.com</t>
+  </si>
+  <si>
+    <t>$2a$12$8Ybnu3VPciLD5s9d507TLejcyGmjm94j2uh5LRMKZ7NfvtgHH1ca2</t>
   </si>
 </sst>
 </file>
@@ -437,13 +449,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" bestFit="true" customWidth="true" width="2.7109375"/>
     <col min="2" max="2" bestFit="true" customWidth="true" width="9.20703125"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="15.23046875"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="65.36328125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="22.92578125"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="63.4765625"/>
     <col min="5" max="5" bestFit="true" customWidth="true" width="10.91015625"/>
   </cols>
   <sheetData>
@@ -498,6 +510,23 @@
         <v>14</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="B4" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="C4" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="D4" t="s" s="0">
+        <v>18</v>
+      </c>
+      <c r="E4" t="s" s="0">
+        <v>14</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
users list get initiated with excel
</commit_message>
<xml_diff>
--- a/App/CLI-backend/databases/UserDatabase.xlsx
+++ b/App/CLI-backend/databases/UserDatabase.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="32">
   <si>
     <t>ID</t>
   </si>
@@ -65,6 +65,57 @@
   </si>
   <si>
     <t>11-09-1100</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>$2a$12$HDQ4cNX2tqwm7mOtB/Ngie0v6R.DBxORQaZUAaapcwKcRf.mgv.bO</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>$2a$12$jZo6Yy0QVVb1PmLBZ1WNZ.sQPMK2Plz.ZbqjN7121wxRQt1vpK4MC</t>
+  </si>
+  <si>
+    <t>5</t>
+  </si>
+  <si>
+    <t>$2a$12$B9pDOoHyeMxnEv/8W93qAeNZWrW2BehCcLjq.DX8CrlBIMLxg0qFu</t>
+  </si>
+  <si>
+    <t>6</t>
+  </si>
+  <si>
+    <t>Serban123</t>
+  </si>
+  <si>
+    <t>2@y.com</t>
+  </si>
+  <si>
+    <t>$2a$12$LEmc/Jt7ZGNXFGtUdp/LI.ND/BIftqlcX00nGu4qkkTWRSRXedNwO</t>
+  </si>
+  <si>
+    <t>30-08-2000</t>
+  </si>
+  <si>
+    <t>7</t>
+  </si>
+  <si>
+    <t>$2a$12$xBjaZf1EvExCIPvl2PZo6.DbGfTkj7VLdmQGfPKt.uGb0Qv97F5T6</t>
+  </si>
+  <si>
+    <t>8</t>
+  </si>
+  <si>
+    <t>$2a$12$CWleeXeQLt2DgQ4ielPv..X4G/lPNgL9Eqo9BOHkuRe./qYGHIDFC</t>
+  </si>
+  <si>
+    <t>9</t>
+  </si>
+  <si>
+    <t>$2a$12$pTI6Arhn2a9Q53zdiblfAu2BYr68N5t07I653hOr.O/Fkw/sq8mFi</t>
   </si>
 </sst>
 </file>
@@ -437,11 +488,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" bestFit="true" customWidth="true" width="2.7109375"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="9.20703125"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="9.7109375"/>
     <col min="3" max="3" bestFit="true" customWidth="true" width="15.23046875"/>
     <col min="4" max="4" bestFit="true" customWidth="true" width="65.36328125"/>
     <col min="5" max="5" bestFit="true" customWidth="true" width="10.91015625"/>
@@ -498,6 +549,125 @@
         <v>14</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="B4" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="C4" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="D4" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="E4" t="s" s="0">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="B5" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="C5" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="D5" t="s" s="0">
+        <v>18</v>
+      </c>
+      <c r="E5" t="s" s="0">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s" s="0">
+        <v>19</v>
+      </c>
+      <c r="B6" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="C6" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="D6" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="E6" t="s" s="0">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="B7" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="C7" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="D7" t="s" s="0">
+        <v>24</v>
+      </c>
+      <c r="E7" t="s" s="0">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s" s="0">
+        <v>26</v>
+      </c>
+      <c r="B8" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="C8" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="D8" t="s" s="0">
+        <v>27</v>
+      </c>
+      <c r="E8" t="s" s="0">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s" s="0">
+        <v>28</v>
+      </c>
+      <c r="B9" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="C9" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="D9" t="s" s="0">
+        <v>29</v>
+      </c>
+      <c r="E9" t="s" s="0">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s" s="0">
+        <v>30</v>
+      </c>
+      <c r="B10" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="C10" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="D10" t="s" s="0">
+        <v>31</v>
+      </c>
+      <c r="E10" t="s" s="0">
+        <v>9</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Created parsers package and started ExcelParser with UserParser
</commit_message>
<xml_diff>
--- a/App/CLI-backend/databases/UserDatabase.xlsx
+++ b/App/CLI-backend/databases/UserDatabase.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DELL\Downloads\ZTH-Team-Deltaspace\App\CLI-backend\databases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD3AA2ED-248E-4D19-BB1F-F5DC9E904FFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C78A6D85-294C-4E67-8CC7-35DBC12456AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
   <si>
     <t>ID</t>
   </si>
@@ -46,7 +46,7 @@
     <t>test@admin</t>
   </si>
   <si>
-    <t>$2a$12$.8f5of5jHYP0IkiHyRvaB.fNCEVGKTM2ZgjeuF/Jd1IVfwFDft0pS</t>
+    <t>$2a$12$gjHVm51ixJlapO/reUNmO.v3l8SSAQ7Y4vADbl0i.ji/PSMsRVAEG</t>
   </si>
   <si>
     <t>01-01-2000</t>
@@ -61,52 +61,10 @@
     <t>mihaiviorelstan@gmail.com</t>
   </si>
   <si>
-    <t>$2a$12$dFXj26exmWO1qy1T8a2BJO1WUG5Bx808hZ.bWQBValcptUoiJYIYu</t>
+    <t>$2a$12$x21oBRHzFm8wgynDXaVhKu43EiOGSSlAPLMMbPbtD67rLG9GjL98S</t>
   </si>
   <si>
     <t>15-05-2004</t>
-  </si>
-  <si>
-    <t>3</t>
-  </si>
-  <si>
-    <t>Mihai12</t>
-  </si>
-  <si>
-    <t>mihaiviis@gmail.com</t>
-  </si>
-  <si>
-    <t>$2a$12$8Ybnu3VPciLD5s9d507TLejcyGmjm94j2uh5LRMKZ7NfvtgHH1ca2</t>
-  </si>
-  <si>
-    <t>4</t>
-  </si>
-  <si>
-    <t>Serban123</t>
-  </si>
-  <si>
-    <t>s@y.com</t>
-  </si>
-  <si>
-    <t>$2a$12$e.OoKtEB9ipvvbtnSkRpTu.CWK64XxuPRjy7Yxa/CoZBLfeAt1zai</t>
-  </si>
-  <si>
-    <t>30-08-2000</t>
-  </si>
-  <si>
-    <t>5</t>
-  </si>
-  <si>
-    <t>Serban12</t>
-  </si>
-  <si>
-    <t>s@ya.com</t>
-  </si>
-  <si>
-    <t>$2a$12$9p3ngfxICKBp6WSmh3Wjt.DzchQDtV6lcUdbW3CVrXoN1QQxTBfMm</t>
-  </si>
-  <si>
-    <t>30-05-2000</t>
   </si>
 </sst>
 </file>
@@ -479,13 +437,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" bestFit="true" customWidth="true" width="2.7109375"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="9.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="9.20703125"/>
     <col min="3" max="3" bestFit="true" customWidth="true" width="22.92578125"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="63.87109375"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="64.77734375"/>
     <col min="5" max="5" bestFit="true" customWidth="true" width="10.91015625"/>
   </cols>
   <sheetData>
@@ -540,57 +498,6 @@
         <v>14</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="s" s="0">
-        <v>15</v>
-      </c>
-      <c r="B4" t="s" s="0">
-        <v>16</v>
-      </c>
-      <c r="C4" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="D4" t="s" s="0">
-        <v>18</v>
-      </c>
-      <c r="E4" t="s" s="0">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="s" s="0">
-        <v>19</v>
-      </c>
-      <c r="B5" t="s" s="0">
-        <v>20</v>
-      </c>
-      <c r="C5" t="s" s="0">
-        <v>21</v>
-      </c>
-      <c r="D5" t="s" s="0">
-        <v>22</v>
-      </c>
-      <c r="E5" t="s" s="0">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="s" s="0">
-        <v>24</v>
-      </c>
-      <c r="B6" t="s" s="0">
-        <v>25</v>
-      </c>
-      <c r="C6" t="s" s="0">
-        <v>26</v>
-      </c>
-      <c r="D6" t="s" s="0">
-        <v>27</v>
-      </c>
-      <c r="E6" t="s" s="0">
-        <v>28</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Basic REST API with users and posts with images.
</commit_message>
<xml_diff>
--- a/App/CLI-backend/databases/UserDatabase.xlsx
+++ b/App/CLI-backend/databases/UserDatabase.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
   <si>
     <t>ID</t>
   </si>
@@ -65,6 +65,21 @@
   </si>
   <si>
     <t>30-08-2000</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>mmmmm213</t>
+  </si>
+  <si>
+    <t>s@yy.com</t>
+  </si>
+  <si>
+    <t>$2a$12$jmwxQzadIykWO2nuswoyVeS7mk3.DAg066p3RKSY69qAL9BVVRcqq</t>
+  </si>
+  <si>
+    <t>30-09-2000</t>
   </si>
 </sst>
 </file>
@@ -437,13 +452,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" bestFit="true" customWidth="true" width="2.7109375"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="9.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="11.40234375"/>
     <col min="3" max="3" bestFit="true" customWidth="true" width="10.53515625"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="63.77734375"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="64.48046875"/>
     <col min="5" max="5" bestFit="true" customWidth="true" width="10.91015625"/>
   </cols>
   <sheetData>
@@ -481,23 +496,6 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="B3" t="s" s="0">
-        <v>11</v>
-      </c>
-      <c r="C3" t="s" s="0">
-        <v>12</v>
-      </c>
-      <c r="D3" t="s" s="0">
-        <v>13</v>
-      </c>
-      <c r="E3" t="s" s="0">
-        <v>14</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Overwrite own folder with App folder.
</commit_message>
<xml_diff>
--- a/App/CLI-backend/databases/UserDatabase.xlsx
+++ b/App/CLI-backend/databases/UserDatabase.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="24">
   <si>
     <t>ID</t>
   </si>
@@ -80,6 +80,18 @@
   </si>
   <si>
     <t>30-09-2000</t>
+  </si>
+  <si>
+    <t>Mihai14</t>
+  </si>
+  <si>
+    <t>mihai@gmail.com</t>
+  </si>
+  <si>
+    <t>$2a$12$qN.3gSO5DDZagJMmw98ayeZMdpkg8svoM4Ngu42ara.01oNbmDWsG</t>
+  </si>
+  <si>
+    <t>15-05-2004</t>
   </si>
 </sst>
 </file>
@@ -452,13 +464,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" bestFit="true" customWidth="true" width="2.7109375"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="11.40234375"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="10.53515625"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="64.48046875"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="9.20703125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="15.23046875"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="65.375"/>
     <col min="5" max="5" bestFit="true" customWidth="true" width="10.91015625"/>
   </cols>
   <sheetData>
@@ -496,6 +508,23 @@
         <v>9</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="B3" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="C3" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="D3" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="E3" t="s" s="0">
+        <v>23</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Post database up and running
</commit_message>
<xml_diff>
--- a/App/CLI-backend/databases/UserDatabase.xlsx
+++ b/App/CLI-backend/databases/UserDatabase.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="31">
   <si>
     <t>ID</t>
   </si>
@@ -92,6 +92,27 @@
   </si>
   <si>
     <t>15-05-2004</t>
+  </si>
+  <si>
+    <t>Mihai12</t>
+  </si>
+  <si>
+    <t>mihaiviorelstan@gmail.com</t>
+  </si>
+  <si>
+    <t>$2a$12$YzZWSJuSyxQx1rw11YlPruJqByi14NSE1.Lel34NnBFws0YmLsrey</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>Mihai16</t>
+  </si>
+  <si>
+    <t>mihai16@gmail.com</t>
+  </si>
+  <si>
+    <t>$2a$12$jqncT20LIoitS7YBDlwA/ufkEftcLETLgvvUjN9BBpk4s.6T79k3O</t>
   </si>
 </sst>
 </file>
@@ -464,12 +485,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" bestFit="true" customWidth="true" width="2.7109375"/>
     <col min="2" max="2" bestFit="true" customWidth="true" width="9.20703125"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="15.23046875"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="22.92578125"/>
     <col min="4" max="4" bestFit="true" customWidth="true" width="65.375"/>
     <col min="5" max="5" bestFit="true" customWidth="true" width="10.91015625"/>
   </cols>
@@ -525,6 +546,40 @@
         <v>23</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="B4" t="s" s="0">
+        <v>24</v>
+      </c>
+      <c r="C4" t="s" s="0">
+        <v>25</v>
+      </c>
+      <c r="D4" t="s" s="0">
+        <v>26</v>
+      </c>
+      <c r="E4" t="s" s="0">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s" s="0">
+        <v>27</v>
+      </c>
+      <c r="B5" t="s" s="0">
+        <v>28</v>
+      </c>
+      <c r="C5" t="s" s="0">
+        <v>29</v>
+      </c>
+      <c r="D5" t="s" s="0">
+        <v>30</v>
+      </c>
+      <c r="E5" t="s" s="0">
+        <v>23</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
changed .gitignore to not commit .env
</commit_message>
<xml_diff>
--- a/App/CLI-backend/databases/UserDatabase.xlsx
+++ b/App/CLI-backend/databases/UserDatabase.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="15">
   <si>
     <t>1</t>
   </si>
@@ -53,6 +53,18 @@
   </si>
   <si>
     <t>$2a$12$Nba9LbbhluPg7MAKtSvXD.9nlG.iY.WecDEQ2baUr0.2i1wG5.bvW</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>Mihai12</t>
+  </si>
+  <si>
+    <t>mihaistan@gmail.com</t>
+  </si>
+  <si>
+    <t>$2a$12$qaqRQWR./udlP/6RlKRh.eATubFWV8mSD75/fF8sSEUL5wLOynFl2</t>
   </si>
 </sst>
 </file>
@@ -425,13 +437,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" bestFit="true" customWidth="true" width="1.9140625"/>
     <col min="2" max="2" bestFit="true" customWidth="true" width="7.2109375"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="15.23046875"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="62.171875"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="18.62890625"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="62.4765625"/>
     <col min="5" max="5" bestFit="true" customWidth="true" width="10.11328125"/>
   </cols>
   <sheetData>
@@ -486,6 +498,23 @@
         <v>4</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="s" s="0">
+        <v>11</v>
+      </c>
+      <c r="B4" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="C4" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="D4" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="E4" t="s" s="0">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>